<commit_message>
Uploading final test results and reports
</commit_message>
<xml_diff>
--- a/src/test/resources/Data.xlsx
+++ b/src/test/resources/Data.xlsx
@@ -51,10 +51,10 @@
     <t>Lal Kothi</t>
   </si>
   <si>
-    <t>online</t>
-  </si>
-  <si>
     <t>Center</t>
+  </si>
+  <si>
+    <t>Online</t>
   </si>
 </sst>
 </file>
@@ -394,7 +394,7 @@
         <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>8</v>
@@ -460,7 +460,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7">
         <v>57809</v>

</xml_diff>